<commit_message>
data updated to 2024
</commit_message>
<xml_diff>
--- a/data/data_2016.xlsx
+++ b/data/data_2016.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/TakumaWatari/Dropbox/Research data/2024/Steel-flows/clean/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/TakumaWatari/Dropbox/GitHub/steel-flows-sankeys/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4DC8BB7-57E8-C240-B7B6-7747E1A15D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4F8500-8291-FB46-83BB-7F76BE1F7CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="840" windowWidth="38400" windowHeight="19560" xr2:uid="{95929309-E14E-F341-94AB-0DA32D6E9E75}"/>
+    <workbookView xWindow="14300" yWindow="-31400" windowWidth="38400" windowHeight="29840" xr2:uid="{95929309-E14E-F341-94AB-0DA32D6E9E75}"/>
   </bookViews>
   <sheets>
     <sheet name="list" sheetId="44" r:id="rId1"/>
@@ -55,7 +55,7 @@
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateCount="1000" iterateDelta="0.01"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -242,8 +242,8 @@
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -510,14 +510,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -6441,21 +6441,21 @@
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="10">
-        <v>1974.1567164179107</v>
+        <v>2126.0149253731347</v>
       </c>
       <c r="G3" s="10">
-        <v>0.89328358208899772</v>
+        <v>0</v>
       </c>
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
       <c r="K3" s="9"/>
       <c r="L3" s="12">
-        <v>1975.0499999999997</v>
+        <v>2126.0149253731347</v>
       </c>
       <c r="M3" s="12"/>
       <c r="N3" s="12">
-        <v>0</v>
+        <v>-150.96492537313497</v>
       </c>
       <c r="O3" s="7">
         <v>537.70499999999993</v>
@@ -6511,21 +6511,21 @@
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="10">
-        <v>1063.0074626865674</v>
+        <v>911.14925373134338</v>
       </c>
       <c r="G5" s="10">
-        <v>1879.5442085809204</v>
+        <v>1880.4374921630094</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
       <c r="K5" s="9"/>
       <c r="L5" s="12">
-        <v>2942.551671267488</v>
+        <v>2791.586745894353</v>
       </c>
       <c r="M5" s="12"/>
       <c r="N5" s="12">
-        <v>1734.9889671962399</v>
+        <v>1885.9538925693748</v>
       </c>
       <c r="O5" s="7">
         <v>57.82</v>

</xml_diff>